<commit_message>
Notes internes masquées par défaut (anti-fuite à l'export)
- AnalyseContent : les sections "interne" (notes de travail avocat) ne sont plus
  rendues par défaut ; elles n'apparaissent qu'en mode interne explicite
  (?interne=1), avec un bandeau d'avertissement. Plus aucune fuite en vue
  normale / impression / capture / partage de lien.
- controle-ecarts.py : le constat "interne" passe en INFO (masqué par défaut),
  avec rappel que le texte reste dans le JSON livré.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/documents/pieces-defense/Consommation-personnel-et-offerts.xlsx
+++ b/public/documents/pieces-defense/Consommation-personnel-et-offerts.xlsx
@@ -779,7 +779,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -878,36 +878,66 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>- Sur-versement au verre (~8 %)</t>
+          <t>- Sur-versement au verre et cocktails (free-pour, Kerr 2008)</t>
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>446</v>
+        <v>807</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
+          <t>- Degustation offerte (pichet + vin nomme au verre)</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>- Cremant jete en fin de journee (eventé)</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="n">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>- Freinte technique de la biere pression (mousse, lignes)</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="n">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
           <t>- Stock final (inventaire)</t>
         </is>
       </c>
-      <c r="B11" s="4" t="n">
+      <c r="B14" s="4" t="n">
         <v>213</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="5">
-        <f> PERTE REELLE RESIDUELLE (22.8 % des achats)</f>
+    <row r="15">
+      <c r="A15" s="5">
+        <f> PERTE REELLE RESIDUELLE (15.9 % des achats)</f>
         <v/>
       </c>
-      <c r="B12" s="6" t="n">
-        <v>2419</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Perte d'exploitation d'un bar (casse, evaporation, mousse, sur-versement non mesure). A rapprocher de l'abattement que l'administration retient elle-meme en reconstitution de bar (CAA Paris, 17 mars 2021 : 22 % des achats pour personnel/offerts/pertes/vol, methode validee ; n de requete a fiabiliser). AUCUNE vente au noir : CA bancarise, especes 1,3 %.</t>
+      <c r="B15" s="6" t="n">
+        <v>1690</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Le residuel est desormais la seule perte IRREDUCTIBLE (casse, evaporation, fonds de verre, rincage) : les autres pertes sont chiffrees en postes explicites. La perte d'exploitation TOTALE (conso personnel + offerts + sur-versement + degustation + cremant + freinte + casse) atteint 28.7 % des achats, AU-DESSUS des 22 % que l'administration retient elle-meme en reconstitution de bar (CAA Paris, 17 mars 2021, methode validee ; n de requete a fiabiliser). AUCUNE vente au noir : CA bancarise, especes 1,3 %.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Pertes bière : tableaux refondus + freinte 20% documentée et sourcée
- Tableau 1 dédupliqué : une ligne par produit (pression, Pinte, Picon, Panaché,
  Pinte Picon, Monaco) avec part bière (cl), qté + L par exercice et total
  (fin des doublons dus aux deux cartes). Total 1 293 L.
- Tableau 2 : freinte technique par exercice, composants en % du fût
  (sur-versement/collerette 7 %, mousse & tirage 8 %, nettoyage + purge + fond
  5 %) = 20 % (323 L), au-dessus des 15 % du fisc.
- Sources citées avec liens : Modern Restaurant Management (moyenne 20 %/fût),
  Bar-i (5-25 %, moussage >10 %), Brewers Association (nettoyage lignes 14 j),
  Le Bihan Boissons (~10 % FR), JDC (~15 % FR).
- Découplage : la cascade « Boissons disparues » garde une freinte prudente de
  10 % (129 L) inchangée (assert + Monte-Carlo intacts) ; phrase de réconciliation.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/documents/pieces-defense/Consommation-personnel-et-offerts.xlsx
+++ b/public/documents/pieces-defense/Consommation-personnel-et-offerts.xlsx
@@ -779,7 +779,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -878,21 +878,21 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>- Sur-versement au verre et cocktails (free-pour, Kerr 2008)</t>
+          <t>- Sur-versement vins/spiritueux/cocktails (free-pour : Kerr 2008, Wansink 2005)</t>
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>807</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>- Degustation offerte (pichet + vin nomme au verre)</t>
+          <t>- Degustation offerte (note par note, annexe C)</t>
         </is>
       </c>
       <c r="B11" s="4" t="n">
-        <v>113</v>
+        <v>126</v>
       </c>
     </row>
     <row r="12">
@@ -902,40 +902,50 @@
         </is>
       </c>
       <c r="B12" s="4" t="n">
-        <v>126</v>
+        <v>260</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>- Freinte technique de la biere pression (mousse, lignes)</t>
+          <t>- Cremant sur-versé (free-pour +23,6 %)</t>
         </is>
       </c>
       <c r="B13" s="4" t="n">
-        <v>129</v>
+        <v>87</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
+          <t>- Freinte technique de la biere pression (mousse, lignes)</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="n">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
           <t>- Stock final (inventaire)</t>
         </is>
       </c>
-      <c r="B14" s="4" t="n">
+      <c r="B15" s="4" t="n">
         <v>213</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="5">
-        <f> PERTE REELLE RESIDUELLE (15.9 % des achats)</f>
+    <row r="16">
+      <c r="A16" s="5">
+        <f> PERTE REELLE RESIDUELLE (11.4 % des achats)</f>
         <v/>
       </c>
-      <c r="B15" s="6" t="n">
-        <v>1690</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="B16" s="6" t="n">
+        <v>1207</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
         <is>
           <t>Le residuel est desormais la seule perte IRREDUCTIBLE (casse, evaporation, fonds de verre, rincage) : les autres pertes sont chiffrees en postes explicites. La perte d'exploitation TOTALE (conso personnel + offerts + sur-versement + degustation + cremant + freinte + casse) atteint 28.7 % des achats, AU-DESSUS des 22 % que l'administration retient elle-meme en reconstitution de bar (CAA Paris, 17 mars 2021, methode validee ; n de requete a fiabiliser). AUCUNE vente au noir : CA bancarise, especes 1,3 %.</t>
         </is>

</xml_diff>

<commit_message>
Pertes bière : contenance verre vs part bière + tailles 25/50 distinctes
- Tableau 1 par ARTICLE de caisse (format_service), tailles 25 et 50 cl
  séparées (Pression 25/50, Picon bière 25/50 ; Panaché et Monaco 25 cl only).
- Deux colonnes distinctes : Contenance verre et Part bière réelle. Parts :
  panaché/monaco 12,5 cl (moitié bière + limonade/grenadine), Picon 23 cl (demi,
  2 cl Picon) / 46 cl (pinte, 4 cl). Part bière totale = 1 219 L (verre 1 293 L).
- Ventilation 25/50 lue sur l'article, insensible aux variations de prix par
  période (note ajoutée).
- Freinte (Table 2) recalculée sur la part bière : 20 % = 305 L. Cascade
  « disparu » inchangée (freinte 129 L, calée sur la contenance verre) : assert
  global et Monte-Carlo intacts.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/documents/pieces-defense/Consommation-personnel-et-offerts.xlsx
+++ b/public/documents/pieces-defense/Consommation-personnel-et-offerts.xlsx
@@ -882,7 +882,7 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>1056</v>
+        <v>1058</v>
       </c>
     </row>
     <row r="11">
@@ -937,11 +937,11 @@
     </row>
     <row r="16">
       <c r="A16" s="5">
-        <f> PERTE REELLE RESIDUELLE (11.4 % des achats)</f>
+        <f> PERTE REELLE RESIDUELLE (11.3 % des achats)</f>
         <v/>
       </c>
       <c r="B16" s="6" t="n">
-        <v>1207</v>
+        <v>1205</v>
       </c>
     </row>
     <row r="18">

</xml_diff>

<commit_message>
Rendu final : mise en page normalisée + refonte page 2.8 (coefficient)
Mise en page (toutes les pages /rendu-final, via scripts/rfcommun.py) :
- conclusion = dernière section titrée, en texte normal (plus de carte verte)
- pièces téléchargeables = simple carte, après la conclusion (plus de gros titre)
- chapitres numérotés séquentiellement ; normaliseur partagé intégré aux 11 générateurs
- liens en violet/italique (distincts du gras) ; notes lisibles ; lead-ins en sous-titres

Page 2.8 (coefficient liquide/solide) réécrite et démontée poste par poste :
- le coefficient EST le ratio solides/liquides de la propre caisse (incohérence interne)
- cuisine fantôme = 354 921 € = 75 % du redressement (écho du gonflement des boissons)
- effet de levier x4 ; cuisine mesurable directement (annexes C), jamais mesurée

Fusion 2.1.a dans 2.6 ; détail menus (proba x dose x vendus) ; 0 tiret cadratin.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/documents/pieces-defense/Consommation-personnel-et-offerts.xlsx
+++ b/public/documents/pieces-defense/Consommation-personnel-et-offerts.xlsx
@@ -882,7 +882,7 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>1058</v>
+        <v>720</v>
       </c>
     </row>
     <row r="11">
@@ -937,11 +937,11 @@
     </row>
     <row r="16">
       <c r="A16" s="5">
-        <f> PERTE REELLE RESIDUELLE (11.3 % des achats)</f>
+        <f> PERTE REELLE RESIDUELLE (14.5 % des achats)</f>
         <v/>
       </c>
       <c r="B16" s="6" t="n">
-        <v>1205</v>
+        <v>1543</v>
       </c>
     </row>
     <row r="18">

</xml_diff>